<commit_message>
docs: bang tong ket sheet 01 ke them Bang 3b cho OnboardingFileSizeBvaTest
Bang 3b khong them test nao — no trinh bay lai 6 test da co san trong
OnboardingFileSizeBvaTest, va 6 test do da nam trong tong 56 tu dau:

  19  RegisterStandardBvaTest
  17  RegisterTagCoverageTest
  14  RegisterEquivalencePartitionTest
   6  OnboardingFileSizeBvaTest   <- chinh la 6 dong cua Bang 3b
  ---
  56

Nhung cot "Thi hanh bang nao" o dong 9 van chi ghi Bang 4 va Bang 5, chua ke
Bang 3b. Doc bang tong ket thi tuong lop nay khong lien quan gi toi Bang 3b,
trong khi Bang 3b chinh la no. Da sua thanh:

  Bang 3b · case 20-25
  Bang 4  · V5, X12, B22-B27
  Bang 5  · TC18-TC23

Dung nhu cach form dang ky duoc trinh bay: 19 test cua no xuat hien o Bang 2 va
3 (dang BVA), Bang 4 (dang nhan), Bang 5 (dang test case gop tag). Cung mot bo
test, ba goc nhin — khong phai ba bo test khac nhau.

399 test, 0 that bai.
</commit_message>
<xml_diff>
--- a/BaoCao-KiemThu-CareerCompass.xlsx
+++ b/BaoCao-KiemThu-CareerCompass.xlsx
@@ -1723,8 +1723,8 @@
     <mergeCell ref="F8:H8"/>
     <mergeCell ref="F17:H17"/>
     <mergeCell ref="F23:H23"/>
+    <mergeCell ref="F28:H28"/>
     <mergeCell ref="F22:H22"/>
-    <mergeCell ref="F28:H28"/>
     <mergeCell ref="F13:H13"/>
     <mergeCell ref="F30:H30"/>
     <mergeCell ref="F9:H9"/>
@@ -10327,7 +10327,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1">
+    <row r="9" ht="44" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>OnboardingFileSizeBvaTest</t>
@@ -10343,7 +10343,8 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Bảng 4 · V5, X12, B22–B27
+          <t>Bảng 3b · case 20–25
+Bảng 4 · V5, X12, B22–B27
 Bảng 5 · TC18–TC23</t>
         </is>
       </c>

</xml_diff>